<commit_message>
Add missing Custom Message, Audio Message test cases to Send Message and Audio Call, Incoming Call test cases to Call Module
</commit_message>
<xml_diff>
--- a/Call_Module/Calls_Module_Test_Cases.xlsx
+++ b/Call_Module/Calls_Module_Test_Cases.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2052,13 +2052,689 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Verify Audio Call</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on a conversation</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Verify initiating an audio call</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>1. Open a one-on-one conversation.
+2. Click the audio call (phone) icon in header.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Audio call should initiate. Calling screen should appear with user name, avatar, and call controls.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call ringing state</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>1. Initiate an audio call to another user.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Ringing state should display with 'Calling...' or ringing indicator. Ring tone should play.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call connected state</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>1. Initiate audio call.
+2. Other user accepts.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Call should connect. Timer should start. Audio should be active both ways.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call mute/unmute</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>1. During an active audio call.
+2. Click mute button.
+3. Click unmute.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Mute should silence outgoing audio. Unmute should restore it. Icon should toggle.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call speaker toggle</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>1. During an active audio call.
+2. Click speaker button.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Audio should switch between earpiece and speaker. Icon should toggle.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Verify ending an audio call</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>1. During an active audio call.
+2. Click end call (red) button.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Call should end. Both users should return to chat. Call duration should log.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call in group</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>1. Open a group conversation.
+2. Initiate an audio call.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Group audio call should initiate. All members should receive call notification.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Verify Audio Call</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call when user is offline</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>1. Try to audio call a user who is offline.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Call should ring and eventually show 'User unavailable' or similar message.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in, network disconnected</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call fails without network</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>1. Disconnect network.
+2. Try to initiate an audio call.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Error message should display indicating no network connection.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr"/>
+      <c r="C53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and on an active call</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio call drops on network loss</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>1. Be on an active audio call.
+2. Disconnect network.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Call should drop with reconnecting attempt or error message.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Verify Incoming Call</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and app is open</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Verify incoming audio call notification</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>1. Another user initiates an audio call to you.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Incoming call screen should appear with caller name, avatar, accept and reject buttons.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Verify incoming video call notification</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>1. Another user initiates a video call to you.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Incoming call screen should appear with caller name, avatar, accept and reject buttons.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Verify accepting an incoming audio call</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>1. Receive an incoming audio call.
+2. Click accept/answer button.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Audio call should connect. Call screen should show with active call controls.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Verify accepting an incoming video call</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>1. Receive an incoming video call.
+2. Click accept/answer button.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Video call should connect with both video feeds visible.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Verify rejecting an incoming call</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>1. Receive an incoming call.
+2. Click reject/decline button.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Call should be rejected. Caller should see 'Call declined' or similar. Call logged as missed.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_058</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr"/>
+      <c r="C59" s="2" t="inlineStr"/>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Verify incoming call when app is in background</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>1. Minimize the app.
+2. Another user calls you.</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Push notification or system call UI should appear allowing accept/reject.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Verify incoming group call notification</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>1. A group member initiates a group call.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Incoming group call notification should appear with group name and accept/reject options.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_060</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" s="2" t="inlineStr"/>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Verify missed call when not answered</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>1. Receive an incoming call.
+2. Do not answer until it times out.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Call should be logged as 'Missed' in call logs. Missed call notification should appear.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Verify Incoming Call</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with Do Not Disturb enabled</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Verify incoming call behavior with DND</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>1. Enable Do Not Disturb.
+2. Receive an incoming call.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Call should be silenced or blocked based on DND settings. Call logged as missed.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>CALLS_062</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr"/>
+      <c r="C63" s="2" t="inlineStr"/>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and already on a call</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Verify incoming call while on another call</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>1. Be on an active call.
+2. Receive another incoming call.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Second call notification should appear with option to accept (end current) or reject.</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="25">
     <mergeCell ref="C42:C43"/>
     <mergeCell ref="B25:B30"/>
     <mergeCell ref="C15:C20"/>
+    <mergeCell ref="B21:B24"/>
     <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B21:B24"/>
     <mergeCell ref="D21:D24"/>
     <mergeCell ref="B42:B43"/>
     <mergeCell ref="D36:D37"/>

</xml_diff>